<commit_message>
Single line Mode translation is working as expected
</commit_message>
<xml_diff>
--- a/demo_impex_bulk_less.xlsx
+++ b/demo_impex_bulk_less.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SanchitSS\impex-studio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7CFAFC2-8D04-42DA-8E0E-DF1C62A926EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF2C9B35-96B9-43FE-B119-136D2B54FB45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A83101BC-ADDE-4993-A06C-F936E110D158}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
   <si>
     <t>content</t>
   </si>
@@ -47,16 +47,7 @@
     <t>OmegaLinkHero</t>
   </si>
   <si>
-    <t>&lt;div class="top-banner-area"&gt; &lt;img class="omegaLink-top-banner-img" src="https://assets.omega.com/landing-pages/omega-link/omegaLink-desktop-hero-bg.png" alt="Omega Link Desktop" width="2160" height="1214"/&gt; &lt;div class="omegaLink-banner-content"&gt; &lt;h1&gt;Omega Link&lt;/h1&gt; &lt;img class="omegaLink-top-banner-img-mobile" src="https://assets.omega.com/landing-pages/omega-link/omegaLink-desktop-hero-bg.png" alt="Omega Link Mobile" width="2160" height="1214"/&gt;&lt;p&gt;Connecting mission-critical sensors and systems&lt;/p&gt;&lt;a href="https://cloud.mail.omega.com/omega-link-consultation" target="_blank" class="omegaLink-btn btn btn-secondary"&gt;Request a Consultation&lt;/a&gt; &lt;/div&gt;&lt;/div&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;&lt;strong&gt; Netherlands 07077 03815 International +31 (0) 7077 03815&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;ukcustomerservice@dwyeromega.com&lt;/strong&gt;&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>QuotePrintPreviewContactNoComponetUS</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;&lt;strong&gt; 1-800-872-9141&lt;/strong&gt; (US &amp; Canada)&lt;/p&gt;&lt;p&gt;&lt;strong&gt;omegainfo@dwyeromega.com&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;casalesinfo@dwyeromega.com&lt;/strong&gt; (for Canada)&lt;/p&gt;</t>
   </si>
   <si>
     <t>OrderPrintPreviewContactNoComponetNL</t>
@@ -65,7 +56,13 @@
     <t>techResourceArticleSignUpComponent</t>
   </si>
   <si>
-    <t>&lt;div class='footer-techResourceArticleSignUp'&gt;&lt;div class='footer-techResourceArticleSignUp-container'&gt;&lt;div class='title'&gt;Technology Club&lt;/div&gt;&lt;div class='footer-techResourceArticleSignUp-copy'&gt;&lt;p&gt;Get our latest articles straight into your inbox!&lt;/p&gt;&lt;a href='https://info.dwyeromega.com/communications-signup' target='_blank' title='Join club' alt='Join club'&gt;Join club&lt;/a&gt;&lt;/div&gt;&lt;/div&gt;&lt;/div&gt;&lt;div class='clearfix'&gt;&lt;/div&gt;</t>
+    <t>&lt;div class='footer-techResourceArticleSignUp'&gt;Welcome "6-66001-2" &lt;/div&gt;</t>
+  </si>
+  <si>
+    <t>&lt;div class="footer-techResourceArticleSignUp"&gt;Welcome "6-66001-2" &lt;/div&gt;</t>
+  </si>
+  <si>
+    <t>&lt;DIV CLASS='footer-techResourceArticleSignUp'&gt;Welcome "6-66001-2"&lt;/DIV&gt;</t>
   </si>
 </sst>
 </file>
@@ -147,13 +144,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -499,43 +496,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="B3" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
+      <c r="B5" s="5" t="s">
         <v>7</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="72" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -571,11 +568,11 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B15" s="5"/>
-      <c r="C15" s="6"/>
+      <c r="C15" s="8"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B16" s="5"/>
-      <c r="C16" s="6"/>
+      <c r="C16" s="8"/>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B17" s="5"/>

</xml_diff>

<commit_message>
Complete app developed for EMEA tanslations
</commit_message>
<xml_diff>
--- a/demo_impex_bulk_less.xlsx
+++ b/demo_impex_bulk_less.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SanchitSS\impex-studio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF2C9B35-96B9-43FE-B119-136D2B54FB45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1A5979A-D32C-42CD-A595-3E8070A0EE96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A83101BC-ADDE-4993-A06C-F936E110D158}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>content</t>
   </si>
@@ -56,13 +56,16 @@
     <t>techResourceArticleSignUpComponent</t>
   </si>
   <si>
-    <t>&lt;div class='footer-techResourceArticleSignUp'&gt;Welcome "6-66001-2" &lt;/div&gt;</t>
-  </si>
-  <si>
-    <t>&lt;div class="footer-techResourceArticleSignUp"&gt;Welcome "6-66001-2" &lt;/div&gt;</t>
-  </si>
-  <si>
-    <t>&lt;DIV CLASS='footer-techResourceArticleSignUp'&gt;Welcome "6-66001-2"&lt;/DIV&gt;</t>
+    <t>&lt;div class="footer-techResourceArticleSignUp"&gt;Welcome "6-66001-2"  &lt;img itemprop="image" title="Ahmar Bajwa" alt="Ahmar Bajwa" src="https://assets.omega.com/landing-pages/meet-team/team-ahmar.png" loading="lazy" width="455" height="454"/&gt;&lt;/div&gt;</t>
+  </si>
+  <si>
+    <t>&lt;DIV CLASS='footer-techResourceArticleSignUp'&gt;Image "6-66001-2"  &lt;img itemprop="image" title="Ahmar Bajwa" alt="Ahmar Bajwa" src="https://assets.omega.com/landing-pages/meet-team/team-ahmar.png" loading="lazy" width="455" height="454"/&gt;&lt;/DIV&gt;</t>
+  </si>
+  <si>
+    <t>&lt;div class="footer-techResourceArticleSignUp"&gt;Cart "6-66001-2"  &lt;img itemprop="image" title="Ahmar Bajwa" alt="Ahmar Bajwa" src="https://assets.omega.com/landing-pages/meet-team/team-ahmar.png" loading="lazy" width="455" height="454"/&gt;&lt;/div&gt;</t>
+  </si>
+  <si>
+    <t>&lt;div class='footer-techResourceArticleSignUp'&gt;Color "6-66001-2"  &lt;img itemprop="image" title="Ahmar Bajwa" alt="Ahmar Bajwa" src="https://assets.omega.com/landing-pages/meet-team/team-ahmar.png" loading="lazy" width="455" height="454"/&gt;&lt;/div&gt;</t>
   </si>
 </sst>
 </file>
@@ -503,36 +506,36 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Single component loader, html UI Done
</commit_message>
<xml_diff>
--- a/demo_impex_bulk_less.xlsx
+++ b/demo_impex_bulk_less.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SanchitSS\impex-studio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1A5979A-D32C-42CD-A595-3E8070A0EE96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FB16664-5A22-4998-91B2-017D60BFBC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A83101BC-ADDE-4993-A06C-F936E110D158}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>content</t>
   </si>
@@ -44,28 +44,34 @@
     <t>component_Id</t>
   </si>
   <si>
-    <t>OmegaLinkHero</t>
-  </si>
-  <si>
-    <t>QuotePrintPreviewContactNoComponetUS</t>
-  </si>
-  <si>
-    <t>OrderPrintPreviewContactNoComponetNL</t>
-  </si>
-  <si>
-    <t>techResourceArticleSignUpComponent</t>
-  </si>
-  <si>
-    <t>&lt;div class="footer-techResourceArticleSignUp"&gt;Welcome "6-66001-2"  &lt;img itemprop="image" title="Ahmar Bajwa" alt="Ahmar Bajwa" src="https://assets.omega.com/landing-pages/meet-team/team-ahmar.png" loading="lazy" width="455" height="454"/&gt;&lt;/div&gt;</t>
-  </si>
-  <si>
-    <t>&lt;DIV CLASS='footer-techResourceArticleSignUp'&gt;Image "6-66001-2"  &lt;img itemprop="image" title="Ahmar Bajwa" alt="Ahmar Bajwa" src="https://assets.omega.com/landing-pages/meet-team/team-ahmar.png" loading="lazy" width="455" height="454"/&gt;&lt;/DIV&gt;</t>
-  </si>
-  <si>
-    <t>&lt;div class="footer-techResourceArticleSignUp"&gt;Cart "6-66001-2"  &lt;img itemprop="image" title="Ahmar Bajwa" alt="Ahmar Bajwa" src="https://assets.omega.com/landing-pages/meet-team/team-ahmar.png" loading="lazy" width="455" height="454"/&gt;&lt;/div&gt;</t>
-  </si>
-  <si>
-    <t>&lt;div class='footer-techResourceArticleSignUp'&gt;Color "6-66001-2"  &lt;img itemprop="image" title="Ahmar Bajwa" alt="Ahmar Bajwa" src="https://assets.omega.com/landing-pages/meet-team/team-ahmar.png" loading="lazy" width="455" height="454"/&gt;&lt;/div&gt;</t>
+    <t>comp_00000335</t>
+  </si>
+  <si>
+    <t>&lt;div class="micable-features"&gt; 		&lt;div class="micable-features-title"&gt; 			&lt;span&gt;5 Unique Features of Omega's MI Cable&lt;/span&gt; 		&lt;/div&gt; 		&lt;div class="micable-features-content"&gt; 			&lt;div class="cable-feature"&gt; 				&lt;img src="https://assets.omega.com/micable/icon-coins.png" width="" height="" class="feature-icon" /&gt; 				&lt;span class="feature-title"&gt;High Purity M&lt;sub&gt;g&lt;/sub&gt;O Insulation&lt;/span&gt; 				&lt;ul&gt; 					&lt;li&gt;Less thermal drift at high temperatures&lt;/li&gt; 					&lt;li&gt;Results in longer probe life and reduced costs&lt;/li&gt; 				&lt;/ul&gt; 			&lt;/div&gt; 			&lt;div class="cable-feature"&gt; 				&lt;img src="https://assets.omega.com/micable/icon-graph.png" width="" height="" class="feature-icon" /&gt; 				&lt;span class="feature-title"&gt;Special Limits of Error (SLE) Standard&lt;/span&gt; 				&lt;ul&gt; 					&lt;li&gt;Increased accuracy for no additional cost&lt;/li&gt; 					&lt;li&gt;Results in higher quality production in critical applications&lt;/li&gt; 				&lt;/ul&gt; 			&lt;/div&gt; 			&lt;div class="cable-feature"&gt; 				&lt;img src="https://assets.omega.com/micable/icon-bell.png " width="" height="" class="feature-icon" /&gt; 				&lt;span class="feature-title"&gt;Special Services&lt;/span&gt; 				&lt;ul&gt; 					&lt;li&gt;Lot thermoelectric properties provided upon request&lt;/li&gt; 					&lt;li&gt;AMS 2750 available; 3' samples at no additional cost&lt;/li&gt; 				&lt;/ul&gt; 			&lt;/div&gt; 			&lt;div class="cable-feature"&gt; 				&lt;img src="https://assets.omega.com/micable/icon-signal.png" width="" height="" class="feature-icon" /&gt; 				&lt;span class="feature-title"&gt;Dual MI Cable&lt;/span&gt; 				&lt;ul&gt; 					&lt;li&gt;Carries two signals for critical applications&lt;/li&gt; 					&lt;li&gt;Saves space and reduces cost when you have to carry multiple signals&lt;/li&gt; 					&lt;li&gt;Provides redundancy for added protection to your process&lt;/li&gt; 				&lt;/ul&gt; 			&lt;/div&gt; 			&lt;div class="cable-feature"&gt; 				&lt;img src="https://assets.omega.com/micable/icon-thermometer.png" width="" height="" class="feature-icon" /&gt; 				&lt;span class="feature-title"&gt;Exclusive XL MI Cable&lt;/span&gt; 				&lt;ul&gt; 					&lt;li&gt;Designed for use at consistently high temperatures&lt;/li&gt; 					&lt;li&gt;Most accurate high temperature thermocouple over time&lt;/li&gt; 					&lt;li&gt;Highest temperature rating of all MI cable&lt;/li&gt; 					&lt;li&gt;Can be used in hydrogen atmospheres&lt;/li&gt; 				&lt;/ul&gt; 			&lt;/div&gt; 		&lt;/div&gt; 	&lt;/div&gt;</t>
+  </si>
+  <si>
+    <t>comp_00000337</t>
+  </si>
+  <si>
+    <t>&lt;div class="micable-hero"&gt;&lt;div class="template-container"&gt;&lt;div class="micable-hero-content"&gt;&lt;h1&gt;HIGH-PERFORMANCE MI CABLE&lt;/h1&gt;&lt;span class="subHead"&gt;Put Our Temperature Expertise to Work for Your Product&lt;/span&gt; 				&lt;span class="subHeadCaption"&gt;Large selection of sheaths, thermocouple types, and diameters.&lt;/span&gt;&lt;/div&gt;&lt;/div&gt;&lt;/div&gt;	&lt;div class="micable-banner"&gt;		&lt;div class="template-container"&gt;			&lt;div class="micable-banner-content"&gt;				&lt;span&gt;AGGRESSIVE OEM PRICING&lt;br&gt; IN STOCK &amp; FAST DELIVERY FOR LARGE VOLUME ORDERS&lt;/span&gt;			&lt;/div&gt;		&lt;/div&gt;	&lt;/div&gt;</t>
+  </si>
+  <si>
+    <t>comp_00000338</t>
+  </si>
+  <si>
+    <t>&lt;div class="micable-form"&gt; &lt;div class="micable-form-title"&gt;Get In Touch With Our Experts Now&lt;/div&gt; &lt;form action="https://omega--OmegaDEV.cs91.my.salesforce.com/servlet/servlet.WebToCase?encoding=UTF-8" method="POST"&gt;     &lt;!--&lt;input type="hidden" name="captcha_settings" value="{&amp;quot;keyname&amp;quot;:&amp;quot;Omega_Global_reCAPTCHA_Key&amp;quot;,&amp;quot;fallback&amp;quot;:&amp;quot;true&amp;quot;,&amp;quot;orgId&amp;quot;:&amp;quot;00D2F0000008qq8&amp;quot;,&amp;quot;ts&amp;quot;:&amp;quot;&amp;quot;}" /&gt;--&gt; &lt;input type="hidden" name="orgid" value="00D2F0000008qq8" /&gt; &lt;input type="hidden" name="retURL" value="https://www.omega.ca/mi-cable" /&gt; &lt;input type="hidden" name="recordType" id="recordType" value="0122F0000004Xjb" /&gt; &lt;input id="recordType" name="recordType" type="hidden" /&gt;  &lt;!--  ----------------------------------------------------------------------  --&gt; &lt;!--  NOTE: These fields are optional debugging elements. Please uncomment    --&gt; &lt;!--  these lines if you wish to test in debug mode.                          --&gt; &lt;!--  &lt;input type="hidden" name="debug" value=1&gt;                              --&gt; &lt;!--  &lt;input type="hidden" name="debugEmail"                                  --&gt; &lt;!--  value="dward@westmonroepartners.com"&gt;                                   --&gt; &lt;!--  ----------------------------------------------------------------------  --&gt;  &lt;label for="00N2F000000hLQk"&gt;First Name*&lt;/label&gt;&lt;input id="00N2F000000hLQk" maxlength="255" name="00N2F000000hLQk" size="20" type="text" required="" /&gt;&lt;br /&gt;     &lt;label for="00N2F000000hLQu"&gt;Last Name*&lt;/label&gt;&lt;input id="00N2F000000hLQu" maxlength="255" name="00N2F000000hLQu" size="20" type="text" required="" /&gt;&lt;br /&gt;     &lt;label for="00N2F000000hLJe"&gt;Job Title*&lt;/label&gt;&lt;input id="00N2F000000hLJe" maxlength="40" name="00N2F000000hLJe" size="20" type="text" required="" /&gt;&lt;br /&gt;     &lt;label for="email"&gt;Email*&lt;/label&gt;&lt;input id="email" maxlength="80" name="email" size="20" type="text" required="" /&gt;&lt;br /&gt;     &lt;label for="phone"&gt;Phone Number*&lt;/label&gt;&lt;input id="phone" maxlength="40" name="phone" size="20" type="text" required="" /&gt;&lt;br /&gt;     &lt;label for="company"&gt;Company&lt;/label&gt;&lt;input id="company" maxlength="80" name="company" size="20" type="text" required="" /&gt;&lt;br /&gt;     &lt;label for="description"&gt;Description&lt;/label&gt;&lt;textarea name="description"&gt;&lt;/textarea&gt;&lt;br /&gt;     &lt;div class="g-recaptcha" data-sitekey="6Lfg3F4UAAAAAAf2wNchL_1qHmBbS6_O9yiXfEEX"&gt;&amp;nbsp;&lt;/div&gt;     &lt;br /&gt;     &lt;input type="submit" name="submit" class="btn btn-primary" /&gt; &lt;/form&gt; &lt;/div&gt;</t>
+  </si>
+  <si>
+    <t>comp_000003V0</t>
+  </si>
+  <si>
+    <t>comp_000003V1</t>
+  </si>
+  <si>
+    <t>&lt;div class="micable-hero-content" style="color:#000"&gt;&lt;h1&gt;This is a test&lt;/h1&gt; This should display on the mi cable page at the bottom.&lt;/div&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &lt;div id="rohsModal" class="modal fade in" aria-hidden="false"&gt; 		&lt;div class="modal-dialog"&gt; 			&lt;div class="modal-content"&gt; 				&lt;div&gt; 					&lt;button type="button" class="close" data-dismiss="modal" id="cboxClose"&gt; 						&lt;img src="https://assets.omega.com/landing-pages/my-x-button.png" alt="Close Button"&gt; 					&lt;/button&gt;  					&lt;p class="modalHeading" style="background-color:#0068b3;border:thick solid #0068b3;"&gt; 						&lt;b&gt;Thank you for your inquiry&lt;/b&gt; 					&lt;/p&gt; 				&lt;/div&gt; 				&lt;div id="loaderDiv"&gt;&lt;img src="/Universal/wwwcore/images/loader.gif" style="display: inline;"&gt;&lt;/div&gt; 				&lt;div class="modalText"&gt; 					First McLast,&lt;br&gt; 					Your form has been submitted successfully and our engineers will be contact you shortly.&lt;br&gt;&lt;br&gt; 					You can &lt;a href="#" id="closeLink"&gt;close this window&lt;/a&gt;, or read more about MI Cables: 					&lt;div class="modalTextArticle"&gt; 					&lt;a href="/resources/what-is-mi-cable" target="_parent" class="modalArticle"&gt; 						&lt;span class="segmentTag techLearning"&gt;Technical Learning&lt;/span&gt; 		                	&lt;img alt="What is MI Cable?" class="categoryArticleImg" width="248" height="150" src="https://assets.omega.com/resources/what-is-mi-cable-uf.jpg"&gt; 					&lt;/a&gt; 					&lt;/div&gt; 				&lt;/div&gt; 			&lt;/div&gt; 		&lt;/div&gt; &lt;/div&gt;	</t>
   </si>
 </sst>
 </file>
@@ -130,7 +136,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -150,7 +156,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -494,7 +499,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="103.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="81.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="112.33203125" style="1" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
   </cols>
   <sheetData>
@@ -506,40 +511,45 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B6" s="5"/>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B7" s="5"/>
@@ -571,11 +581,11 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B15" s="5"/>
-      <c r="C15" s="8"/>
+      <c r="C15" s="7"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B16" s="5"/>
-      <c r="C16" s="8"/>
+      <c r="C16" s="7"/>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B17" s="5"/>

</xml_diff>